<commit_message>
Daily recap, matchup updates, learning and research 2026-08-18
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-18.xlsx
+++ b/data/k-props/2026-08-18.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="102">
   <si>
     <t>date</t>
   </si>
@@ -145,6 +145,9 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -160,16 +163,25 @@
     <t>St. Louis Cardinals @ Cincinnati Reds</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>&lt;6</t>
   </si>
   <si>
     <t>Kyle Leahy</t>
   </si>
   <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>Carson Whisenhunt</t>
   </si>
   <si>
     <t>San Francisco Giants @ Cleveland Guardians</t>
+  </si>
+  <si>
+    <t>U</t>
   </si>
   <si>
     <t>Foster Griffin</t>
@@ -886,17 +898,23 @@
       <c r="Y2">
         <v>1.0455</v>
       </c>
+      <c r="Z2">
+        <v>10</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>0.63</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>6.13</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.2019</v>
@@ -906,6 +924,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>3.87</v>
+      </c>
+      <c r="AJ2">
+        <v>3.87</v>
+      </c>
+      <c r="AK2">
+        <v>3.87</v>
+      </c>
+      <c r="AL2">
+        <v>3.87</v>
       </c>
       <c r="AM2">
         <v>6.13</v>
@@ -916,7 +946,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -931,28 +961,28 @@
         <v>41</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L3">
         <v>6</v>
       </c>
       <c r="S3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:39" x14ac:dyDescent="0.25">
@@ -960,7 +990,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4">
         <v>4.5</v>
@@ -972,7 +1002,7 @@
         <v>-126</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G4">
         <v>824475</v>
@@ -1031,17 +1061,23 @@
       <c r="Y4">
         <v>0.9052</v>
       </c>
+      <c r="Z4">
+        <v>6</v>
+      </c>
       <c r="AA4" t="s">
         <v>44</v>
       </c>
+      <c r="AB4">
+        <v>-1.09</v>
+      </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="AD4">
         <v>3.41</v>
       </c>
       <c r="AE4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF4">
         <v>0.166</v>
@@ -1051,6 +1087,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>2.59</v>
+      </c>
+      <c r="AJ4">
+        <v>2.59</v>
+      </c>
+      <c r="AK4">
+        <v>2.59</v>
+      </c>
+      <c r="AL4">
+        <v>2.59</v>
       </c>
       <c r="AM4">
         <v>3.41</v>
@@ -1061,7 +1109,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>5.5</v>
@@ -1073,7 +1121,7 @@
         <v>-120</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G5">
         <v>824475</v>
@@ -1132,17 +1180,23 @@
       <c r="Y5">
         <v>1.0796</v>
       </c>
+      <c r="Z5">
+        <v>6</v>
+      </c>
       <c r="AA5" t="s">
         <v>44</v>
       </c>
+      <c r="AB5">
+        <v>1.29</v>
+      </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD5">
         <v>6.79</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.2328</v>
@@ -1152,6 +1206,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>-0.79</v>
+      </c>
+      <c r="AJ5">
+        <v>0.79</v>
+      </c>
+      <c r="AK5">
+        <v>-0.79</v>
+      </c>
+      <c r="AL5">
+        <v>0.79</v>
       </c>
       <c r="AM5">
         <v>6.79</v>
@@ -1162,7 +1228,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C6">
         <v>3.5</v>
@@ -1174,7 +1240,7 @@
         <v>-107</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G6">
         <v>824398</v>
@@ -1233,17 +1299,23 @@
       <c r="Y6">
         <v>0.9198</v>
       </c>
+      <c r="Z6">
+        <v>1</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB6">
+        <v>-0.4</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
         <v>3.1</v>
       </c>
       <c r="AE6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF6">
         <v>0.1754</v>
@@ -1253,6 +1325,18 @@
       </c>
       <c r="AH6">
         <v>0</v>
+      </c>
+      <c r="AI6">
+        <v>-2.1</v>
+      </c>
+      <c r="AJ6">
+        <v>2.1</v>
+      </c>
+      <c r="AK6">
+        <v>-2.1</v>
+      </c>
+      <c r="AL6">
+        <v>2.1</v>
       </c>
       <c r="AM6">
         <v>3.1</v>
@@ -1263,7 +1347,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C7">
         <v>5.5</v>
@@ -1275,7 +1359,7 @@
         <v>-105</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G7">
         <v>824398</v>
@@ -1334,17 +1418,23 @@
       <c r="Y7">
         <v>1.0041</v>
       </c>
+      <c r="Z7">
+        <v>6</v>
+      </c>
       <c r="AA7" t="s">
         <v>44</v>
       </c>
+      <c r="AB7">
+        <v>-0.94</v>
+      </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="AD7">
         <v>4.56</v>
       </c>
       <c r="AE7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF7">
         <v>0.1877</v>
@@ -1354,6 +1444,18 @@
       </c>
       <c r="AH7">
         <v>0</v>
+      </c>
+      <c r="AI7">
+        <v>1.44</v>
+      </c>
+      <c r="AJ7">
+        <v>1.44</v>
+      </c>
+      <c r="AK7">
+        <v>1.44</v>
+      </c>
+      <c r="AL7">
+        <v>1.44</v>
       </c>
       <c r="AM7">
         <v>4.56</v>
@@ -1364,7 +1466,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C8">
         <v>3.5</v>
@@ -1376,7 +1478,7 @@
         <v>122</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>823341</v>
@@ -1435,17 +1537,23 @@
       <c r="Y8">
         <v>1.0856</v>
       </c>
+      <c r="Z8">
+        <v>3</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB8">
+        <v>0.99</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="AD8">
         <v>4.49</v>
       </c>
       <c r="AE8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF8">
         <v>0.1563</v>
@@ -1455,6 +1563,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>-1.49</v>
+      </c>
+      <c r="AJ8">
+        <v>1.49</v>
+      </c>
+      <c r="AK8">
+        <v>-1.49</v>
+      </c>
+      <c r="AL8">
+        <v>1.49</v>
       </c>
       <c r="AM8">
         <v>4.49</v>
@@ -1465,7 +1585,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>5.5</v>
@@ -1477,7 +1597,7 @@
         <v>104</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>823341</v>
@@ -1536,17 +1656,23 @@
       <c r="Y9">
         <v>0.8825</v>
       </c>
+      <c r="Z9">
+        <v>4</v>
+      </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB9">
+        <v>-0.64</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD9">
         <v>4.86</v>
       </c>
       <c r="AE9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF9">
         <v>0.2588</v>
@@ -1556,6 +1682,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>-0.86</v>
+      </c>
+      <c r="AJ9">
+        <v>0.86</v>
+      </c>
+      <c r="AK9">
+        <v>-0.86</v>
+      </c>
+      <c r="AL9">
+        <v>0.86</v>
       </c>
       <c r="AM9">
         <v>4.86</v>
@@ -1566,7 +1704,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C10">
         <v>7.5</v>
@@ -1578,7 +1716,7 @@
         <v>-136</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G10">
         <v>823423</v>
@@ -1637,17 +1775,23 @@
       <c r="Y10">
         <v>0.8983</v>
       </c>
+      <c r="Z10">
+        <v>7</v>
+      </c>
       <c r="AA10" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB10">
+        <v>-0.97</v>
       </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD10">
         <v>6.53</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.2988</v>
@@ -1657,6 +1801,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>0.47</v>
+      </c>
+      <c r="AJ10">
+        <v>0.47</v>
+      </c>
+      <c r="AK10">
+        <v>0.47</v>
+      </c>
+      <c r="AL10">
+        <v>0.47</v>
       </c>
       <c r="AM10">
         <v>6.53</v>
@@ -1667,7 +1823,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C11">
         <v>4.5</v>
@@ -1679,31 +1835,31 @@
         <v>-142</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L11">
         <v>6</v>
       </c>
       <c r="S11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.25">
@@ -1711,7 +1867,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C12">
         <v>3.5</v>
@@ -1723,7 +1879,7 @@
         <v>-136</v>
       </c>
       <c r="F12" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G12">
         <v>822938</v>
@@ -1782,17 +1938,23 @@
       <c r="Y12">
         <v>0.9953</v>
       </c>
+      <c r="Z12">
+        <v>5</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>-0.63</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD12">
         <v>2.87</v>
       </c>
       <c r="AE12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF12">
         <v>0.1366</v>
@@ -1802,6 +1964,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>2.13</v>
+      </c>
+      <c r="AJ12">
+        <v>2.13</v>
+      </c>
+      <c r="AK12">
+        <v>2.13</v>
+      </c>
+      <c r="AL12">
+        <v>2.13</v>
       </c>
       <c r="AM12">
         <v>2.87</v>
@@ -1812,7 +1986,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C13">
         <v>3.5</v>
@@ -1824,7 +1998,7 @@
         <v>110</v>
       </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G13">
         <v>824723</v>
@@ -1883,17 +2057,23 @@
       <c r="Y13">
         <v>0.9954</v>
       </c>
+      <c r="Z13">
+        <v>2</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB13">
+        <v>-0.19</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD13">
         <v>3.31</v>
       </c>
       <c r="AE13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF13">
         <v>0.1621</v>
@@ -1903,6 +2083,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>-1.31</v>
+      </c>
+      <c r="AJ13">
+        <v>1.31</v>
+      </c>
+      <c r="AK13">
+        <v>-1.31</v>
+      </c>
+      <c r="AL13">
+        <v>1.31</v>
       </c>
       <c r="AM13">
         <v>3.31</v>
@@ -1913,7 +2105,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C14">
         <v>4.5</v>
@@ -1925,7 +2117,7 @@
         <v>-105</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G14">
         <v>824723</v>
@@ -1984,17 +2176,23 @@
       <c r="Y14">
         <v>0.88</v>
       </c>
+      <c r="Z14">
+        <v>3</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB14">
+        <v>0.68</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD14">
         <v>5.18</v>
       </c>
       <c r="AE14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF14">
         <v>0.2375</v>
@@ -2004,6 +2202,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>-2.18</v>
+      </c>
+      <c r="AJ14">
+        <v>2.18</v>
+      </c>
+      <c r="AK14">
+        <v>-2.18</v>
+      </c>
+      <c r="AL14">
+        <v>2.18</v>
       </c>
       <c r="AM14">
         <v>5.18</v>
@@ -2014,7 +2224,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2026,7 +2236,7 @@
         <v>100</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G15">
         <v>823586</v>
@@ -2085,17 +2295,23 @@
       <c r="Y15">
         <v>0.9557</v>
       </c>
+      <c r="Z15">
+        <v>4</v>
+      </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB15">
+        <v>0.45</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD15">
         <v>4.95</v>
       </c>
       <c r="AE15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF15">
         <v>0.2051</v>
@@ -2105,6 +2321,18 @@
       </c>
       <c r="AH15">
         <v>0</v>
+      </c>
+      <c r="AI15">
+        <v>-0.95</v>
+      </c>
+      <c r="AJ15">
+        <v>0.95</v>
+      </c>
+      <c r="AK15">
+        <v>-0.95</v>
+      </c>
+      <c r="AL15">
+        <v>0.95</v>
       </c>
       <c r="AM15">
         <v>4.95</v>
@@ -2115,7 +2343,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C16">
         <v>3.5</v>
@@ -2127,31 +2355,31 @@
         <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L16">
         <v>6</v>
       </c>
       <c r="S16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:39" x14ac:dyDescent="0.25">
@@ -2159,7 +2387,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C17">
         <v>4.5</v>
@@ -2171,7 +2399,7 @@
         <v>-106</v>
       </c>
       <c r="F17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G17">
         <v>823667</v>
@@ -2230,17 +2458,23 @@
       <c r="Y17">
         <v>0.9597</v>
       </c>
+      <c r="Z17">
+        <v>3</v>
+      </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB17">
+        <v>0.35</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD17">
         <v>4.85</v>
       </c>
       <c r="AE17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF17">
         <v>0.2536</v>
@@ -2250,6 +2484,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>-1.85</v>
+      </c>
+      <c r="AJ17">
+        <v>1.85</v>
+      </c>
+      <c r="AK17">
+        <v>-1.85</v>
+      </c>
+      <c r="AL17">
+        <v>1.85</v>
       </c>
       <c r="AM17">
         <v>4.85</v>
@@ -2260,7 +2506,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C18">
         <v>4.5</v>
@@ -2272,7 +2518,7 @@
         <v>-123</v>
       </c>
       <c r="F18" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G18">
         <v>823667</v>
@@ -2331,17 +2577,23 @@
       <c r="Y18">
         <v>0.9903</v>
       </c>
+      <c r="Z18">
+        <v>4</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB18">
+        <v>0.82</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="AD18">
         <v>5.32</v>
       </c>
       <c r="AE18" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF18">
         <v>0.2013</v>
@@ -2351,6 +2603,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>-1.32</v>
+      </c>
+      <c r="AJ18">
+        <v>1.32</v>
+      </c>
+      <c r="AK18">
+        <v>-1.32</v>
+      </c>
+      <c r="AL18">
+        <v>1.32</v>
       </c>
       <c r="AM18">
         <v>5.32</v>
@@ -2361,7 +2625,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C19">
         <v>3.5</v>
@@ -2373,31 +2637,31 @@
         <v>130</v>
       </c>
       <c r="F19" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L19">
         <v>3</v>
       </c>
       <c r="S19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.25">
@@ -2405,7 +2669,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C20">
         <v>5.5</v>
@@ -2417,7 +2681,7 @@
         <v>135</v>
       </c>
       <c r="F20" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G20">
         <v>823749</v>
@@ -2476,17 +2740,23 @@
       <c r="Y20">
         <v>1.0058</v>
       </c>
+      <c r="Z20">
+        <v>8</v>
+      </c>
       <c r="AA20" t="s">
         <v>44</v>
       </c>
+      <c r="AB20">
+        <v>-0.03</v>
+      </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD20">
         <v>5.47</v>
       </c>
       <c r="AE20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF20">
         <v>0.2938</v>
@@ -2496,6 +2766,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>2.53</v>
+      </c>
+      <c r="AJ20">
+        <v>2.53</v>
+      </c>
+      <c r="AK20">
+        <v>2.53</v>
+      </c>
+      <c r="AL20">
+        <v>2.53</v>
       </c>
       <c r="AM20">
         <v>5.47</v>
@@ -2506,7 +2788,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C21">
         <v>5.5</v>
@@ -2518,7 +2800,7 @@
         <v>-154</v>
       </c>
       <c r="F21" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G21">
         <v>823749</v>
@@ -2577,17 +2859,23 @@
       <c r="Y21">
         <v>1.0453</v>
       </c>
+      <c r="Z21">
+        <v>3</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB21">
+        <v>-0.15</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD21">
         <v>5.35</v>
       </c>
       <c r="AE21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF21">
         <v>0.2207</v>
@@ -2597,6 +2885,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>-2.35</v>
+      </c>
+      <c r="AJ21">
+        <v>2.35</v>
+      </c>
+      <c r="AK21">
+        <v>-2.35</v>
+      </c>
+      <c r="AL21">
+        <v>2.35</v>
       </c>
       <c r="AM21">
         <v>5.35</v>
@@ -2607,7 +2907,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C22">
         <v>6.5</v>
@@ -2619,7 +2919,7 @@
         <v>-138</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G22">
         <v>824639</v>
@@ -2678,17 +2978,23 @@
       <c r="Y22">
         <v>1.0865</v>
       </c>
+      <c r="Z22">
+        <v>5</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB22">
+        <v>-0.4</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD22">
         <v>6.1</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2168</v>
@@ -2698,6 +3004,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>-1.1</v>
+      </c>
+      <c r="AJ22">
+        <v>1.1</v>
+      </c>
+      <c r="AK22">
+        <v>-1.1</v>
+      </c>
+      <c r="AL22">
+        <v>1.1</v>
       </c>
       <c r="AM22">
         <v>6.1</v>
@@ -2708,7 +3026,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C23">
         <v>3.5</v>
@@ -2720,7 +3038,7 @@
         <v>100</v>
       </c>
       <c r="F23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G23">
         <v>822859</v>
@@ -2779,17 +3097,23 @@
       <c r="Y23">
         <v>0.989</v>
       </c>
+      <c r="Z23">
+        <v>5</v>
+      </c>
       <c r="AA23" t="s">
         <v>44</v>
       </c>
+      <c r="AB23">
+        <v>-0.07</v>
+      </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>3.43</v>
       </c>
       <c r="AE23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF23">
         <v>0.1733</v>
@@ -2799,6 +3123,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>1.57</v>
+      </c>
+      <c r="AJ23">
+        <v>1.57</v>
+      </c>
+      <c r="AK23">
+        <v>1.57</v>
+      </c>
+      <c r="AL23">
+        <v>1.57</v>
       </c>
       <c r="AM23">
         <v>3.43</v>
@@ -2809,7 +3145,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C24">
         <v>4.5</v>
@@ -2821,31 +3157,34 @@
         <v>-153</v>
       </c>
       <c r="F24" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L24">
         <v>6</v>
       </c>
       <c r="S24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V24" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="Z24">
+        <v>3</v>
       </c>
       <c r="AA24" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:39" x14ac:dyDescent="0.25">
@@ -2853,7 +3192,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C25">
         <v>4.5</v>
@@ -2865,31 +3204,34 @@
         <v>-150</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L25">
         <v>6</v>
       </c>
       <c r="S25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V25" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="Z25">
+        <v>7</v>
       </c>
       <c r="AA25" t="s">
         <v>44</v>
       </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:39" x14ac:dyDescent="0.25">
@@ -2897,7 +3239,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C26">
         <v>4.5</v>
@@ -2909,13 +3251,13 @@
         <v>-106</v>
       </c>
       <c r="F26" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G26">
         <v>824154</v>
       </c>
       <c r="H26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I26">
         <v>3.9</v>
@@ -2968,17 +3310,23 @@
       <c r="Y26">
         <v>0.9877</v>
       </c>
+      <c r="Z26">
+        <v>5</v>
+      </c>
       <c r="AA26" t="s">
         <v>44</v>
       </c>
+      <c r="AB26">
+        <v>-1.91</v>
+      </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="AD26">
         <v>2.59</v>
       </c>
       <c r="AE26" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF26">
         <v>0.1531</v>
@@ -2988,6 +3336,18 @@
       </c>
       <c r="AH26">
         <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>2.41</v>
+      </c>
+      <c r="AJ26">
+        <v>2.41</v>
+      </c>
+      <c r="AK26">
+        <v>2.41</v>
+      </c>
+      <c r="AL26">
+        <v>2.41</v>
       </c>
       <c r="AM26">
         <v>2.59</v>
@@ -2998,7 +3358,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C27">
         <v>3.5</v>
@@ -3010,7 +3370,7 @@
         <v>-141</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G27">
         <v>824319</v>
@@ -3069,17 +3429,23 @@
       <c r="Y27">
         <v>0.9839</v>
       </c>
+      <c r="Z27">
+        <v>3</v>
+      </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB27">
+        <v>-0.82</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD27">
         <v>2.68</v>
       </c>
       <c r="AE27" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF27">
         <v>0.1458</v>
@@ -3089,6 +3455,18 @@
       </c>
       <c r="AH27">
         <v>0</v>
+      </c>
+      <c r="AI27">
+        <v>0.32</v>
+      </c>
+      <c r="AJ27">
+        <v>0.32</v>
+      </c>
+      <c r="AK27">
+        <v>0.32</v>
+      </c>
+      <c r="AL27">
+        <v>0.32</v>
       </c>
       <c r="AM27">
         <v>2.68</v>
@@ -3099,7 +3477,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C28">
         <v>3.5</v>
@@ -3111,7 +3489,7 @@
         <v>108</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G28">
         <v>824319</v>
@@ -3170,17 +3548,23 @@
       <c r="Y28">
         <v>1.0214</v>
       </c>
+      <c r="Z28">
+        <v>6</v>
+      </c>
       <c r="AA28" t="s">
         <v>44</v>
       </c>
+      <c r="AB28">
+        <v>0.22</v>
+      </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD28">
         <v>3.72</v>
       </c>
       <c r="AE28" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF28">
         <v>0.1555</v>
@@ -3190,6 +3574,18 @@
       </c>
       <c r="AH28">
         <v>0</v>
+      </c>
+      <c r="AI28">
+        <v>2.28</v>
+      </c>
+      <c r="AJ28">
+        <v>2.28</v>
+      </c>
+      <c r="AK28">
+        <v>2.28</v>
+      </c>
+      <c r="AL28">
+        <v>2.28</v>
       </c>
       <c r="AM28">
         <v>3.72</v>
@@ -3200,7 +3596,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F29" t="s">
         <v>41</v>
@@ -3263,16 +3659,16 @@
         <v>1.0725</v>
       </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD29">
         <v>7.38</v>
       </c>
       <c r="AE29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AF29">
         <v>0.2735</v>
@@ -3292,10 +3688,10 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F30" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G30">
         <v>822938</v>
@@ -3355,16 +3751,16 @@
         <v>0.88</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD30">
         <v>3.68</v>
       </c>
       <c r="AE30" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF30">
         <v>0.2197</v>
@@ -3384,16 +3780,16 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F31" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G31">
         <v>823423</v>
       </c>
       <c r="H31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="I31">
         <v>4.5</v>
@@ -3435,16 +3831,16 @@
         <v>0.9664</v>
       </c>
       <c r="AA31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD31">
         <v>2.94</v>
       </c>
       <c r="AE31" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF31">
         <v>0.1859</v>
@@ -3464,10 +3860,10 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F32" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G32">
         <v>823586</v>
@@ -3527,16 +3923,16 @@
         <v>1.0025</v>
       </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD32">
         <v>2.74</v>
       </c>
       <c r="AE32" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF32">
         <v>0.1509</v>
@@ -3556,16 +3952,16 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F33" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G33">
         <v>824075</v>
       </c>
       <c r="H33" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I33">
         <v>2.3</v>
@@ -3619,16 +4015,16 @@
         <v>0.924</v>
       </c>
       <c r="AA33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD33">
         <v>1.75</v>
       </c>
       <c r="AE33" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF33">
         <v>0.2027</v>
@@ -3648,16 +4044,16 @@
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F34" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G34">
         <v>824075</v>
       </c>
       <c r="H34" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I34">
         <v>2</v>
@@ -3711,16 +4107,16 @@
         <v>1.0036</v>
       </c>
       <c r="AA34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD34">
         <v>1.77</v>
       </c>
       <c r="AE34" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF34">
         <v>0.2019</v>
@@ -3740,16 +4136,16 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F35" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G35">
         <v>824639</v>
       </c>
       <c r="H35" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I35">
         <v>1.2</v>
@@ -3803,16 +4199,16 @@
         <v>0.889</v>
       </c>
       <c r="AA35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD35">
         <v>1.08</v>
       </c>
       <c r="AE35" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AF35">
         <v>0.2257</v>

</xml_diff>